<commit_message>
feat(framework): Update automation test framework
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/login_testdata.xlsx
+++ b/src/test/resources/testData/login_testdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tuyen_2251061919\Nam4\DATN\opencart-automation-framework\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C00BF6EA-D042-4637-93C7-B17664E17B86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB0872A5-82A6-4BD6-904B-DECC0B78AFA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Email</t>
   </si>
@@ -33,20 +33,38 @@
     <t>Password</t>
   </si>
   <si>
+    <t>anhnt@gmail.com</t>
+  </si>
+  <si>
     <t>Aa123456</t>
   </si>
   <si>
-    <t>anhnt@gmail.com</t>
-  </si>
-  <si>
-    <t>ngocanh@gmail.com</t>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Expected Error Field</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>LG_02</t>
+  </si>
+  <si>
+    <t>LG_03</t>
+  </si>
+  <si>
+    <t>tester1tt@gmail.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -66,6 +84,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -75,7 +100,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -83,13 +108,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -370,34 +414,56 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultColWidth="22.77734375" defaultRowHeight="18" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="16384" width="22.77734375" style="1"/>
+    <col min="1" max="1" width="10.88671875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="26.33203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="32.33203125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="35.88671875" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="22.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2">
+        <v>123456</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>3</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>